<commit_message>
v1: Update the screenplay
</commit_message>
<xml_diff>
--- a/v1/screenplay.xlsx
+++ b/v1/screenplay.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\develop\self_playing_ruler\v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0A90D2-C98E-44D9-8660-C9CE9DC17964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D22C2C-54B2-4CAC-9AEF-5EA5B415E941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25840" windowHeight="13920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="封标" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="257">
   <si>
     <t>​​画面描述 (分镜)​​</t>
   </si>
@@ -71,16 +71,7 @@
     <t>演示曲目待定</t>
   </si>
   <si>
-    <t>拨动钢尺，用手机测量频率</t>
-  </si>
-  <si>
-    <t>添加一个麦克风，使用程序控制拨动钢尺的不同长度，对麦克风采集到的音频进行傅里叶变换，得到频率。最终拟合出一个高精度的频率-步数(step)函数</t>
-  </si>
-  <si>
     <t>相应的画面（快放）</t>
-  </si>
-  <si>
-    <t>既然为了调音增加了麦克风硬件，那为什么不物尽其用呢？esp32s3开发板刚好有usb接口，可以集成一个usb麦克风，用来录音。</t>
   </si>
   <si>
     <t>原理图/pcb</t>
@@ -3757,41 +3748,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>左半屏：慢速演奏-&gt;快速
-右半屏：问题依次浮现：速度慢</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>左半屏：视频展示
-右半屏：问题依次浮现：线太乱</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>速度太慢，如果调快速度就变成这样了！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>左半屏：弹奏一个音+手机fft，浮现文字：误差xxx
-右半屏：问题依次浮现：音不准</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>左半屏：展示一个串口谱子
-右半屏：问题依次浮现：交互难</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>使用开发连线，实在太乱了</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>此前录制的慢放视频（使用类似进度条的东西，显示每部分时间占用）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>首先是速度问题，拆解一下当前演奏一个音符的流程：
-抬起舵机--&gt;移动钢尺--&gt;舵机按下--&gt;舵机拨动
-其中舵机抬起与落下耗时最多，需要着重优化</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -3801,23 +3758,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>大舵机图片
-三角动效，配上不同的器件</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>音不准，偏差有x.x%，如果偏差超过3%（50音分）就是明显不准了</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>麦克风--&gt;正弦信号-(fft)-&gt;频率图</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>麦克风--&gt;开发板-(usb线)-&gt;mic--电脑</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>继承上面的图
 麦克风--&gt;开发板-(usb线)-&gt;mic--&gt;电脑
                                     -&gt;midi--&gt;</t>
@@ -3829,20 +3769,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>最后，用一个电路板把元件整合起来</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>为了更方便复刻，就只使用成品模块了</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>在屏幕前打一个响指，PCB出现在桌面</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>几个焊接特写（焊接排母亲、安装元件）
-成品效果</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -3892,12 +3819,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>让他们组一个文具乐队！！！
-不过上面这些还没有实现，如果这类视频观众朋友门喜欢，点个关注呦！！
-后续会持续更新的！！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>虽然只有一个乐器，也可以用多个组成不同声部
 接下来就以一首《卡农》作为结尾</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -3923,11 +3844,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>接下来就要注入灵魂，撸代码！！！
-在写了亿点点代码，解决了亿点点bug之后，终于</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>制作过程</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -3936,10 +3852,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>原型机效果</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>引入</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -3949,10 +3861,6 @@
   </si>
   <si>
     <t>片头</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>我一个程序员，让我弹钢尺，他能弹么？弹不了！“没那个能力知道吧”</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -3974,12 +3882,123 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>钢尺琴插入电源、插入数据线，调音（如果时间长就快进）
+mid键盘插入数据线
+打开宿主软件（先配置好，最小化），选择xxx设备
+使用MIDI键盘弹奏一小段音乐《欢乐颂》</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>早年在b站看大佬用钢尺演奏太酷了！我也要！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>电视台停播图</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>哔~</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>哆啦A梦掏出：钢尺</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>那就…上！科！技！
+“自动演奏的钢尺”</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>加加鸽</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>手绘设计图展示
+每个器件特写气泡（根据口播节奏依次出现）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>演奏《哆啦A梦》</t>
+  </si>
+  <si>
+    <t>（华强买瓜语音）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>当前滑块特写
+光驱内部结构特写</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>连线图待绘制</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>仿赛博朋克2077的字体：CyberRuler 2025</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>封面</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>钢尺琴钢尺震动的画面</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>标题</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>赛 博 钢 尺——DIY自动演奏的钢尺</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>首先想到的就是加快按压钢尺的动作，更换更快速的舵机
+要压住钢尺，要有足够的下压力，并且体积不能太大
+但发现不同的电机：速度快、力量大、体积小是一个</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>不可能三角</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，最多只能取其二，其中：
+sg90舵机，力量大、体积小、速度慢
+foc无刷电机，速度快、体积小，力量小
+3D打印机常用的42步进电机，速度快、力量大、体积大</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>拨动钢尺，用手机测量频率
+频率-长度表</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>麦克风--&gt;正弦信号-(fft)-&gt;频率图
+频率-步进表</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>演奏《卡农》
-配上字幕：
+配上字幕滚动：
 软件开发：加加鸽
 硬件开发：加加鸽
 结构建模：加加鸽
@@ -3989,175 +4008,199 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>钢尺琴插入电源、插入数据线，调音（如果时间长就快进）
-mid键盘插入数据线
-打开宿主软件（先配置好，最小化），选择xxx设备
-使用MIDI键盘弹奏一小段音乐《欢乐颂》</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>发现问题</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>早年在b站看大佬用钢尺演奏太酷了！我也要！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>电视台停播图</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>哔~</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>​弹钢尺的画面不变 + ​​​范大将军</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>哆啦A梦掏出：钢尺</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>那就…上！科！技！
-“自动演奏的钢尺”</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>加加鸽</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>手绘设计图展示
-每个器件特写气泡（根据口播节奏依次出现）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>演奏前：来看看效果吧！
-演奏到最后：方案可行！！！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>演奏《哆啦A梦》</t>
-  </si>
-  <si>
-    <t>钢尺琴全屏-(动画)-&gt;半屏</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>不过这样的效果是不能让我满意的，还有很多问题要解决</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>串口一个个发送音符演奏，("5#.", 1)即表示高音升Sol，时长为一拍
-每首歌都要一个音一个音来写，太麻烦了！！！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>首先想到的就是加快按压钢尺的动作，更换更快速的舵机
-要压住钢尺，要有足够的下压力，并且体积不能太大
-但发现不同的电机：速度快、力量大、体积小是一个不可能三角，最多只能取其二，其中：
-sg90舵机，力量大、体积小、速度慢
-foc无刷电机，速度快、体积小，力量小
-3D打印机常用的42步进电机，速度快、力量大、体积大</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>给一个问号
+    <t>发现问题
+优化设计</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>​弹钢尺的画面不变
+范大将军片段</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>我一个程序员，让我弹钢尺，他能弹么？弹不了！
+“没那个能力知道吧”</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>大舵机图片
+不同的器件 + 雷达图（三个维度）动效</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>另外，滑块直接套在丝杆上，阻力比较大，也会影响速度
+光驱中就有导轨的，新设计加上导轨减小阻力也是很必要的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+慢速演奏（正常）
+快速（无法压住钢尺，节奏乱掉）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>首先就是演奏速度
+慢速演奏完：这样已经是极限了
+如果调快速度就变成这样了！！这限制了它演奏很多快节奏的曲目</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>那么，拆解一下当前演奏一个音符的流程：
+抬起舵机--&gt;移动钢尺--&gt;舵机按下--&gt;舵机拨动
+其中舵机抬起与落下耗时最多，需要着重优化</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>我：那怎么办呢？
+刘华强：那，吸铁石
+我：钢尺嘛，可以用电磁铁来吸住他
+我：还挺牢固的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
 《华强买瓜》——吸铁石
-电磁铁吸住钢尺特写（尝试拨动，如果不行就静态展示）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>（华强买瓜语音）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>我：那怎么办呢？
-刘华强：那，吸铁石</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>当前滑块特写
-光驱内部结构特写</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>另外，滑块直接套在丝杆上，阻力比较大，也会影响速度
-光驱中就是有导轨的，新设计加上导轨减小阻力也是必要的</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>其次，就要优化音准。此前调音是通过在桌面测试了几个长度的音高，换算出频率-长度函数。但这样人工测量非常耗时，而且并不准确</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>如发送音符、存储乐谱呢？
-主流的电子乐器都支持midi，所以决定使用usb midi，这样即解决了音符发送的问题，也解决了乐谱存储的问题</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>连线图</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>连线图待绘制</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>这里要不要使用虚拟形象？？？（参考“新石器公园”）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>虚拟形象对话？
-废弃的3d打印件
-100多个commit屏幕滚动</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>AI：等等，这么复杂的工程你一次就成功了？
+电磁铁吸住钢尺特写（尝试拨动，如果不行就静态展示）
+solidworks中4电磁铁+钢尺模型图</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+弹奏一个音+手机fft，浮现文字：误差xxx</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>其次是音不准的问题
+偏差有x.x%，如果偏差超过3%（50音分）就是明显跑调了</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>此前调音是通过在桌面测试了几个长度的音高，拟合出频率-长度函数。演奏的时候通过目标频率换算出具体长度。但这样人工测量非常耗时，而且并不准确</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>因此，需要添加一个麦克风，使用程序控制拨动钢尺的不同长度，对麦克风采集到的音频进行傅里叶变换，得到频率。最终就可以拟合出一个高精度的频率-步进(step)曲线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>既然为了调音增加了麦克风硬件，那为什么不物尽其用呢？
+esp32s3开发板刚好有usb接口，可以集成一个usb麦克风，用来录音。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+麦克风--&gt;开发板-(usb线)-&gt;mic--电脑</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+展示一个串口谱子</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>主流的电子乐器都支持midi，所以决定使用usb midi，这样直接使用编曲软件存midi即可</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>还有一个问题，如何存储乐谱呢？
+此前用串口发送一个音符演奏一个音符，谱子格式是自定义的：
+比如，("5#.", 1)：即表示高音升Sol，时长为一拍
+这样，虽然调试方便，但每首歌都要一个音一个音来写，太麻烦了！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>最后，使用面包板，各种连线实在太乱了
+移动的时候不小心还会碰掉</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>开发板乱糟糟的连线
+拿起连断线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>那么，应该画一个电路板，把元件整合起来</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>连线图
+外面一个框浮现</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI：等等，这么顺利？一次就成功了？
 我：这不是考虑到观众老爷的观看体验，将中间的调试过程压缩了么
 我：结构上迭代设计了很多版
 我：代码也是改了很多次，这里有100多个commit</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>仿赛博朋克2077的字体：CyberRuler 2025</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>封面</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>钢尺琴钢尺震动的画面</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>标题</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>赛 博 钢 尺——DIY自动演奏的钢尺</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">midi键盘演示强弱
-演示效果器
-</t>
+    <t>AI虚拟形象
+口播出镜
+废弃的3d打印件
+100多个commit屏幕滚动</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>方案可行！！！
+不过这样的效果是不能让我满意的，还有很多问题要解决，主要是原型机嘛，一切都是从简的，既然验证思路方向没有问题，那就要完善起来了</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>演奏前：来看看效果吧！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>口播出镜
+演奏《哆啦A梦》</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>接下来就要注入灵魂，撸代码！！！</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>在写了亿点点代码，解决了亿点点bug之后，终于</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>王刚出菜BGM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>为了更方便复刻，就只使用成品模块</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>几个焊接特写（焊接排母、安装元件）
+成品效果</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>何同学5G下载BGM</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>由于有mic，还可以对声音进行一些处理：
 比如对强弱的支持
-添加一些效果器
-甚至你还可以把他当作一个麦克风
-刚刚这句就是用自带的麦克风录制的！</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>分析解决问题</t>
+你还可以添加一些效果器
+甚至你还可以把他当作一个麦克风</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>不同力度弹奏midi键盘演示强弱
+演示效果器（片头cyberpunk 2077 预告BGM）
+口播出镜</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>让他们组一个文具乐队！！！
+不过上面这些还没有实现，如果这类视频观众老爷们喜欢，点个关注呦！！
+后续会持续更新的！！</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -4278,7 +4321,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -4299,19 +4342,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -4381,7 +4411,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4421,16 +4451,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4439,7 +4466,7 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4460,28 +4487,7 @@
     <xf numFmtId="21" fontId="8" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="21" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4489,6 +4495,45 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="45" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4769,28 +4814,28 @@
   <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="35" t="s">
-        <v>250</v>
+      <c r="A1" s="27" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="3" t="s">
-        <v>249</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="3" t="s">
-        <v>251</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="35" t="s">
-        <v>252</v>
+      <c r="A5" s="27" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="3" t="s">
-        <v>253</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -4801,10 +4846,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr defaultColWidth="9.08203125" defaultRowHeight="16.5"/>
   <cols>
-    <col min="1" max="3" width="8.25" style="9" customWidth="1"/>
+    <col min="1" max="2" width="8.25" style="9" customWidth="1"/>
+    <col min="3" max="3" width="8.25" style="40" customWidth="1"/>
     <col min="4" max="5" width="62.83203125" style="9" customWidth="1"/>
     <col min="6" max="6" width="26.25" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.33203125" style="9" customWidth="1"/>
@@ -4816,10 +4862,10 @@
         <v>7</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>190</v>
+        <v>173</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>0</v>
@@ -4841,17 +4887,17 @@
       <c r="B2" s="8">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>213</v>
+      <c r="C2" s="39" t="s">
+        <v>193</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="F2" s="9" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -4862,14 +4908,14 @@
         <f>B2+A2</f>
         <v>1.1574074074074073E-4</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>212</v>
+      <c r="C3" s="39" t="s">
+        <v>192</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>229</v>
+        <v>204</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>6</v>
@@ -4883,14 +4929,14 @@
         <f>B3+A3</f>
         <v>1.7361111111111109E-4</v>
       </c>
-      <c r="C4" s="29" t="s">
-        <v>211</v>
+      <c r="C4" s="28" t="s">
+        <v>191</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -4903,25 +4949,30 @@
       </c>
       <c r="C5" s="30"/>
       <c r="D5" s="9" t="s">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
+      <c r="A6" s="7">
+        <v>0</v>
+      </c>
+      <c r="B6" s="8">
+        <f>B3+A3</f>
+        <v>1.7361111111111109E-4</v>
+      </c>
       <c r="C6" s="30"/>
       <c r="D6" s="9" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="9" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="33">
       <c r="A7" s="7">
         <v>0</v>
       </c>
@@ -4931,443 +4982,450 @@
       </c>
       <c r="C7" s="30"/>
       <c r="D7" s="9" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="33">
       <c r="A8" s="7"/>
       <c r="B8" s="8"/>
-      <c r="C8" s="31"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="9" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>228</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="12" customFormat="1" ht="49.5">
       <c r="A9" s="7"/>
       <c r="B9" s="8"/>
-      <c r="C9" s="29" t="s">
-        <v>209</v>
+      <c r="C9" s="28" t="s">
+        <v>190</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>230</v>
+        <v>205</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
     </row>
-    <row r="10" spans="1:7" s="22" customFormat="1" ht="33">
-      <c r="A10" s="24"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>184</v>
-      </c>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+    <row r="10" spans="1:7" s="21" customFormat="1" ht="33">
+      <c r="A10" s="23"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>170</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="G10" s="20"/>
     </row>
     <row r="11" spans="1:7" ht="33">
       <c r="A11" s="7"/>
       <c r="B11" s="8"/>
-      <c r="C11" s="8" t="s">
-        <v>210</v>
-      </c>
+      <c r="C11" s="29"/>
       <c r="D11" s="9" t="s">
-        <v>219</v>
+        <v>247</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" ht="49.5">
       <c r="A12" s="7"/>
       <c r="B12" s="8"/>
-      <c r="C12" s="29" t="s">
-        <v>222</v>
+      <c r="C12" s="31" t="s">
+        <v>219</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>234</v>
+        <v>220</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>245</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="14"/>
     </row>
-    <row r="13" spans="1:7" ht="33">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" s="15" t="s">
+    <row r="13" spans="1:7" s="19" customFormat="1" ht="49.5">
+      <c r="A13" s="35"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="F13" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="G13" s="17"/>
+    </row>
+    <row r="14" spans="1:7" s="19" customFormat="1" ht="49.5">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+    </row>
+    <row r="15" spans="1:7" s="19" customFormat="1" ht="115.5">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+    </row>
+    <row r="16" spans="1:7" s="19" customFormat="1" ht="66">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="G16" s="16"/>
+    </row>
+    <row r="17" spans="1:7" s="19" customFormat="1" ht="33">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+    </row>
+    <row r="18" spans="1:7" ht="33">
+      <c r="A18" s="7"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+    </row>
+    <row r="19" spans="1:7" ht="49.5">
+      <c r="C19" s="33"/>
+      <c r="D19" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="49.5">
+      <c r="C20" s="33"/>
+      <c r="D20" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="22" customFormat="1" ht="33">
+      <c r="A21" s="17"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="16" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" spans="1:7" ht="66">
+      <c r="A22" s="7"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" ht="49.5">
+      <c r="C23" s="33"/>
+      <c r="D23" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="19" customFormat="1" ht="33">
+      <c r="A24" s="35"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>239</v>
+      </c>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+    </row>
+    <row r="25" spans="1:7" s="19" customFormat="1" ht="33">
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="16" t="s">
+        <v>242</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="F25" s="16"/>
+      <c r="G25" s="26" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="C26" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E26" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="F13" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="G13" s="11"/>
-    </row>
-    <row r="14" spans="1:7" ht="33">
-      <c r="A14" s="7"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="E14" s="15" t="s">
+    </row>
+    <row r="27" spans="1:7">
+      <c r="C27" s="33"/>
+      <c r="D27" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="C28" s="33"/>
+      <c r="D28" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="33">
+      <c r="C29" s="33"/>
+      <c r="D29" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="F29" s="10"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="C30" s="33"/>
+      <c r="D30" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="10"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="C31" s="33"/>
+      <c r="D31" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="10"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="C32" s="33"/>
+      <c r="D32" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F32" s="10"/>
+    </row>
+    <row r="33" spans="3:7" ht="33">
+      <c r="C33" s="33"/>
+      <c r="D33" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="10"/>
+    </row>
+    <row r="34" spans="3:7">
+      <c r="C34" s="33"/>
+      <c r="D34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7">
+      <c r="C35" s="33"/>
+      <c r="D35" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="F35" s="10"/>
+    </row>
+    <row r="36" spans="3:7">
+      <c r="C36" s="32"/>
+      <c r="D36" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="37" spans="3:7" ht="66">
+      <c r="C37" s="31" t="s">
+        <v>188</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="38" spans="3:7">
+      <c r="C38" s="33"/>
+      <c r="D38" s="9" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="39" spans="3:7" ht="66">
+      <c r="C39" s="33"/>
+      <c r="D39" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="G39" s="10"/>
+    </row>
+    <row r="40" spans="3:7" ht="66">
+      <c r="C40" s="32"/>
+      <c r="D40" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="41" spans="3:7">
+      <c r="C41" s="31" t="s">
+        <v>187</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="42" spans="3:7">
+      <c r="C42" s="33"/>
+      <c r="D42" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="43" spans="3:7" ht="33">
+      <c r="C43" s="33"/>
+      <c r="D43" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="E43" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-    </row>
-    <row r="15" spans="1:7" ht="33">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>235</v>
-      </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-    </row>
-    <row r="16" spans="1:7" ht="33">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>175</v>
-      </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-    </row>
-    <row r="17" spans="1:7" s="20" customFormat="1" ht="49.5">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="26" t="s">
+    </row>
+    <row r="44" spans="3:7" ht="49.5">
+      <c r="C44" s="32"/>
+      <c r="D44" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-    </row>
-    <row r="18" spans="1:7" s="20" customFormat="1" ht="115.5">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>236</v>
-      </c>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-    </row>
-    <row r="19" spans="1:7" s="20" customFormat="1" ht="49.5">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>238</v>
-      </c>
-      <c r="G19" s="17"/>
-    </row>
-    <row r="20" spans="1:7" s="20" customFormat="1" ht="33">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-    </row>
-    <row r="21" spans="1:7" ht="33">
-      <c r="C21" s="28"/>
-      <c r="D21" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="49.5">
-      <c r="C22" s="28"/>
-      <c r="D22" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" s="23" customFormat="1" ht="33">
-      <c r="A23" s="18"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="E23" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-    </row>
-    <row r="24" spans="1:7" ht="49.5">
-      <c r="C24" s="28"/>
-      <c r="D24" s="9" t="s">
+    </row>
+    <row r="45" spans="3:7" ht="33">
+      <c r="C45" s="31" t="s">
+        <v>186</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E45" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="E24" s="9" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" s="20" customFormat="1">
-      <c r="A25" s="17"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="17" t="s">
-        <v>244</v>
-      </c>
-      <c r="E25" s="17" t="s">
+      <c r="F45" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="F25" s="17"/>
-      <c r="G25" s="34" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="C26" s="26" t="s">
-        <v>208</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="C27" s="28"/>
-      <c r="D27" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="C28" s="28"/>
-      <c r="D28" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="33">
-      <c r="C29" s="28"/>
-      <c r="D29" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="F29" s="10"/>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="C30" s="28"/>
-      <c r="D30" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F30" s="10"/>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="C31" s="28"/>
-      <c r="D31" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="10"/>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="C32" s="28"/>
-      <c r="D32" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F32" s="10"/>
-    </row>
-    <row r="33" spans="3:7" ht="33">
-      <c r="C33" s="28"/>
-      <c r="D33" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="10"/>
-    </row>
-    <row r="34" spans="3:7">
-      <c r="C34" s="28"/>
-      <c r="D34" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="F34" s="10"/>
-    </row>
-    <row r="35" spans="3:7" ht="33">
-      <c r="C35" s="27"/>
-      <c r="D35" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="36" spans="3:7" ht="66">
-      <c r="C36" s="26" t="s">
-        <v>206</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="37" spans="3:7">
-      <c r="C37" s="28"/>
-      <c r="D37" s="9" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="3:7" ht="66">
-      <c r="C38" s="28"/>
-      <c r="D38" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="39" spans="3:7" ht="82.5">
-      <c r="C39" s="27"/>
-      <c r="D39" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="40" spans="3:7">
-      <c r="C40" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="41" spans="3:7">
-      <c r="C41" s="28"/>
-      <c r="D41" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="42" spans="3:7" ht="33">
-      <c r="C42" s="28"/>
-      <c r="D42" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="43" spans="3:7" ht="49.5">
-      <c r="C43" s="27"/>
-      <c r="D43" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="44" spans="3:7" ht="33">
-      <c r="C44" s="26" t="s">
-        <v>204</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="45" spans="3:7" ht="132">
-      <c r="C45" s="27"/>
-      <c r="D45" s="9" t="s">
-        <v>220</v>
+    </row>
+    <row r="46" spans="3:7" ht="132">
+      <c r="C46" s="32"/>
+      <c r="D46" s="9" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="C9:C10"/>
+  <mergeCells count="7">
     <mergeCell ref="C4:C8"/>
-    <mergeCell ref="C12:C16"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="C40:C43"/>
-    <mergeCell ref="C36:C39"/>
-    <mergeCell ref="C26:C35"/>
-    <mergeCell ref="C17:C25"/>
+    <mergeCell ref="C45:C46"/>
+    <mergeCell ref="C41:C44"/>
+    <mergeCell ref="C37:C40"/>
+    <mergeCell ref="C26:C36"/>
+    <mergeCell ref="C12:C25"/>
+    <mergeCell ref="C9:C11"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5387,733 +5445,733 @@
   <sheetData>
     <row r="1" spans="1:7" ht="33">
       <c r="A1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="99">
       <c r="A2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="49.5">
       <c r="A3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="49.5">
       <c r="A4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="E4" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="49.5">
       <c r="A5" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="66">
       <c r="A6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="66">
       <c r="A7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="66">
       <c r="A8" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="33">
       <c r="A9" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="34" t="s">
         <v>98</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="C10" s="34" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="32" t="s">
+      <c r="D10" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="E10" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="F10" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="G10" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="E10" s="32" t="s">
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="34"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="34"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="34"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="B15" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="32"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="32"/>
-      <c r="D11" s="4" t="s">
+      <c r="E15" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="F15" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="G15" s="34" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="34"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="32"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="32"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="32"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="4" t="s">
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="34"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="32"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="4" t="s">
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="34"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="32"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E15" s="32" t="s">
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+    </row>
+    <row r="19" spans="1:7" ht="33">
+      <c r="A19" s="34"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="34"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="32" t="s">
+      <c r="B21" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="E21" s="34" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="32"/>
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="32"/>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="32"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="4" t="s">
+      <c r="F21" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="G21" s="34" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="34"/>
+      <c r="B22" s="34"/>
+      <c r="C22" s="34"/>
+      <c r="D22" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="32"/>
-    </row>
-    <row r="19" spans="1:7" ht="33">
-      <c r="A19" s="32"/>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="4" t="s">
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="34"/>
+      <c r="B23" s="34"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
+    </row>
+    <row r="24" spans="1:7" ht="33">
+      <c r="A24" s="34"/>
+      <c r="B24" s="34"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="32"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32"/>
-      <c r="D20" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" s="32" t="s">
-        <v>115</v>
-      </c>
-      <c r="F21" s="32" t="s">
-        <v>116</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="32"/>
-      <c r="B22" s="32"/>
-      <c r="C22" s="32"/>
-      <c r="D22" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="32"/>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="32"/>
-      <c r="B23" s="32"/>
-      <c r="C23" s="32"/>
-      <c r="D23" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="E23" s="32"/>
-      <c r="F23" s="32"/>
-      <c r="G23" s="32"/>
-    </row>
-    <row r="24" spans="1:7" ht="33">
-      <c r="A24" s="32"/>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
     </row>
     <row r="25" spans="1:7" ht="33">
       <c r="A25" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>122</v>
       </c>
       <c r="E25" s="4"/>
       <c r="F25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="33">
+      <c r="A26" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="E26" s="34" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="33">
-      <c r="A26" s="32" t="s">
+      <c r="F26" s="34" t="s">
         <v>125</v>
       </c>
-      <c r="B26" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="C26" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="G26" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="E26" s="32" t="s">
+    </row>
+    <row r="27" spans="1:7" ht="33">
+      <c r="A27" s="34"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="F26" s="32" t="s">
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="34"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="G26" s="32" t="s">
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="34" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="33">
-      <c r="A27" s="32"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="4" t="s">
+      <c r="B29" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D29" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E27" s="32"/>
-      <c r="F27" s="32"/>
-      <c r="G27" s="32"/>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" s="32"/>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="4" t="s">
+      <c r="E29" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="32" t="s">
+      <c r="F29" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="G29" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="E29" s="32" t="s">
+    </row>
+    <row r="30" spans="1:7" ht="33">
+      <c r="A30" s="34"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="F29" s="32" t="s">
-        <v>135</v>
-      </c>
-      <c r="G29" s="32" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="33">
-      <c r="A30" s="32"/>
-      <c r="B30" s="32"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
     </row>
     <row r="31" spans="1:7" ht="49.5">
       <c r="A31" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C31" s="4" t="s">
+      <c r="F31" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="G31" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="E31" s="4" t="s">
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="34" t="s">
         <v>141</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="B32" s="34" t="s">
         <v>142</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="C32" s="34" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="32" t="s">
+      <c r="D32" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B32" s="32" t="s">
+      <c r="E32" s="34" t="s">
         <v>145</v>
       </c>
-      <c r="C32" s="32" t="s">
+      <c r="F32" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="G32" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="E32" s="32" t="s">
+    </row>
+    <row r="33" spans="1:7" ht="33">
+      <c r="A33" s="34"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="34"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="F32" s="32" t="s">
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="34"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="34"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="34"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="G32" s="32" t="s">
+      <c r="B39" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="C39" s="34" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="33">
-      <c r="A33" s="32"/>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="32"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="32"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="4" t="s">
+      <c r="D39" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="32"/>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="4" t="s">
+      <c r="E39" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="F39" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="G39" s="34" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="34"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="34"/>
+      <c r="D40" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="32"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="4" t="s">
+      <c r="E40" s="34"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="34"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="34"/>
+      <c r="B41" s="34"/>
+      <c r="C41" s="34"/>
+      <c r="D41" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E37" s="32"/>
-      <c r="F37" s="32"/>
-      <c r="G37" s="32"/>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="32"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32"/>
-      <c r="D38" s="4" t="s">
+      <c r="E41" s="34"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="34"/>
+    </row>
+    <row r="42" spans="1:7" ht="33">
+      <c r="A42" s="34"/>
+      <c r="B42" s="34"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="34"/>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="34" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" s="34" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="E43" s="34" t="s">
+        <v>159</v>
+      </c>
+      <c r="F43" s="34" t="s">
+        <v>160</v>
+      </c>
+      <c r="G43" s="34" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="34"/>
+      <c r="B44" s="34"/>
+      <c r="C44" s="34"/>
+      <c r="D44" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E38" s="32"/>
-      <c r="F38" s="32"/>
-      <c r="G38" s="32"/>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="B39" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="C39" s="32" t="s">
-        <v>153</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E39" s="32" t="s">
-        <v>155</v>
-      </c>
-      <c r="F39" s="32" t="s">
-        <v>156</v>
-      </c>
-      <c r="G39" s="32" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="32"/>
-      <c r="B40" s="32"/>
-      <c r="C40" s="32"/>
-      <c r="D40" s="4" t="s">
+      <c r="E44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="34"/>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="34"/>
+      <c r="B45" s="34"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E40" s="32"/>
-      <c r="F40" s="32"/>
-      <c r="G40" s="32"/>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="32"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="4" t="s">
+      <c r="E45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34"/>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="34"/>
+      <c r="B46" s="34"/>
+      <c r="C46" s="34"/>
+      <c r="D46" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="32"/>
-    </row>
-    <row r="42" spans="1:7" ht="33">
-      <c r="A42" s="32"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" s="32" t="s">
-        <v>159</v>
-      </c>
-      <c r="B43" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="C43" s="32" t="s">
-        <v>160</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E43" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="F43" s="32" t="s">
-        <v>163</v>
-      </c>
-      <c r="G43" s="32" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44" s="32"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" s="32"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32"/>
-      <c r="D45" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="E45" s="32"/>
-      <c r="F45" s="32"/>
-      <c r="G45" s="32"/>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" s="32"/>
-      <c r="B46" s="32"/>
-      <c r="C46" s="32"/>
-      <c r="D46" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E46" s="32"/>
-      <c r="F46" s="32"/>
-      <c r="G46" s="32"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="48">

</xml_diff>